<commit_message>
fix bug with signed immmidiate to addiu
</commit_message>
<xml_diff>
--- a/scripts/mips32_r2000_instruction_set.xlsx
+++ b/scripts/mips32_r2000_instruction_set.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="74">
   <si>
     <t>Table 1</t>
   </si>
@@ -94,6 +94,9 @@
     <t>addiu</t>
   </si>
   <si>
+    <t>`EXT_ZERO</t>
+  </si>
+  <si>
     <t>addu</t>
   </si>
   <si>
@@ -109,9 +112,6 @@
     <t>c</t>
   </si>
   <si>
-    <t>`EXT_ZERO</t>
-  </si>
-  <si>
     <t>beq</t>
   </si>
   <si>
@@ -137,6 +137,9 @@
   </si>
   <si>
     <t>jr</t>
+  </si>
+  <si>
+    <t>0</t>
   </si>
   <si>
     <t>`SpecialOP_JR</t>
@@ -1954,7 +1957,7 @@
         <v>25</v>
       </c>
       <c r="M5" t="s" s="16">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="N5" t="s" s="16">
         <v>21</v>
@@ -1965,7 +1968,7 @@
     </row>
     <row r="6" ht="19.5" customHeight="1">
       <c r="A6" t="s" s="14">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B6" s="15">
         <v>0</v>
@@ -2012,7 +2015,7 @@
     </row>
     <row r="7" ht="19.5" customHeight="1">
       <c r="A7" t="s" s="14">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B7" s="15">
         <v>0</v>
@@ -2051,7 +2054,7 @@
         <v>20</v>
       </c>
       <c r="N7" t="s" s="16">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="O7" t="s" s="13">
         <v>22</v>
@@ -2059,10 +2062,10 @@
     </row>
     <row r="8" ht="19.5" customHeight="1">
       <c r="A8" t="s" s="14">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B8" t="s" s="18">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s" s="16">
         <v>17</v>
@@ -2095,10 +2098,10 @@
         <v>25</v>
       </c>
       <c r="M8" t="s" s="16">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="N8" t="s" s="16">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="O8" t="s" s="13">
         <v>22</v>
@@ -2311,21 +2314,37 @@
       <c r="F13" s="17">
         <v>1</v>
       </c>
-      <c r="G13" s="16"/>
-      <c r="H13" s="22"/>
-      <c r="I13" s="22"/>
-      <c r="J13" s="22"/>
-      <c r="K13" s="22"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="22"/>
-      <c r="N13" s="11"/>
+      <c r="G13" t="s" s="16">
+        <v>42</v>
+      </c>
+      <c r="H13" s="17">
+        <v>0</v>
+      </c>
+      <c r="I13" s="17">
+        <v>0</v>
+      </c>
+      <c r="J13" s="17">
+        <v>0</v>
+      </c>
+      <c r="K13" s="17">
+        <v>0</v>
+      </c>
+      <c r="L13" t="s" s="16">
+        <v>19</v>
+      </c>
+      <c r="M13" s="17">
+        <v>0</v>
+      </c>
+      <c r="N13" t="s" s="11">
+        <v>39</v>
+      </c>
       <c r="O13" t="s" s="13">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" ht="19.5" customHeight="1">
       <c r="A14" t="s" s="14">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B14" s="15">
         <v>24</v>
@@ -2352,7 +2371,7 @@
     </row>
     <row r="15" ht="19.5" customHeight="1">
       <c r="A15" t="s" s="14">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B15" s="15">
         <v>25</v>
@@ -2379,7 +2398,7 @@
     </row>
     <row r="16" ht="19.5" customHeight="1">
       <c r="A16" t="s" s="14">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B16" s="15">
         <v>30</v>
@@ -2406,10 +2425,10 @@
     </row>
     <row r="17" ht="19.5" customHeight="1">
       <c r="A17" t="s" s="14">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B17" t="s" s="18">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C17" t="s" s="16">
         <v>17</v>
@@ -2433,7 +2452,7 @@
     </row>
     <row r="18" ht="19.5" customHeight="1">
       <c r="A18" t="s" s="14">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B18" s="15">
         <v>23</v>
@@ -2460,7 +2479,7 @@
     </row>
     <row r="19" ht="19.5" customHeight="1">
       <c r="A19" t="s" s="14">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B19" s="15">
         <v>0</v>
@@ -2499,13 +2518,13 @@
         <v>20</v>
       </c>
       <c r="N19" t="s" s="16">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="O19" s="13"/>
     </row>
     <row r="20" ht="19.5" customHeight="1">
       <c r="A20" t="s" s="14">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B20" s="15">
         <v>0</v>
@@ -2544,16 +2563,16 @@
         <v>20</v>
       </c>
       <c r="N20" t="s" s="16">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="O20" s="13"/>
     </row>
     <row r="21" ht="19.5" customHeight="1">
       <c r="A21" t="s" s="14">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B21" t="s" s="18">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C21" t="s" s="16">
         <v>17</v>
@@ -2586,16 +2605,16 @@
         <v>25</v>
       </c>
       <c r="M21" t="s" s="16">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="N21" t="s" s="16">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="O21" s="13"/>
     </row>
     <row r="22" ht="19.5" customHeight="1">
       <c r="A22" t="s" s="14">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B22" s="15">
         <v>0</v>
@@ -2607,7 +2626,7 @@
         <v>17</v>
       </c>
       <c r="E22" t="s" s="16">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F22" s="22"/>
       <c r="G22" s="22"/>
@@ -2622,10 +2641,10 @@
     </row>
     <row r="23" ht="19.5" customHeight="1">
       <c r="A23" t="s" s="14">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B23" t="s" s="18">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C23" t="s" s="16">
         <v>17</v>
@@ -2649,10 +2668,10 @@
     </row>
     <row r="24" ht="19.5" customHeight="1">
       <c r="A24" t="s" s="14">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B24" t="s" s="18">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C24" t="s" s="16">
         <v>17</v>
@@ -2676,7 +2695,7 @@
     </row>
     <row r="25" ht="19.5" customHeight="1">
       <c r="A25" t="s" s="14">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B25" s="15">
         <v>0</v>
@@ -2688,7 +2707,7 @@
         <v>17</v>
       </c>
       <c r="E25" t="s" s="16">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F25" s="22"/>
       <c r="G25" s="22"/>
@@ -2703,7 +2722,7 @@
     </row>
     <row r="26" ht="19.5" customHeight="1">
       <c r="A26" t="s" s="14">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B26" s="15">
         <v>0</v>
@@ -2742,13 +2761,13 @@
         <v>20</v>
       </c>
       <c r="N26" t="s" s="16">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="O26" s="13"/>
     </row>
     <row r="27" ht="19.5" customHeight="1">
       <c r="A27" t="s" s="14">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B27" s="15">
         <v>0</v>
@@ -2787,13 +2806,13 @@
         <v>20</v>
       </c>
       <c r="N27" t="s" s="16">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="O27" s="13"/>
     </row>
     <row r="28" ht="19.5" customHeight="1">
       <c r="A28" t="s" s="14">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B28" s="15">
         <v>28</v>
@@ -2820,7 +2839,7 @@
     </row>
     <row r="29" ht="19.5" customHeight="1">
       <c r="A29" t="s" s="14">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B29" s="15">
         <v>38</v>
@@ -2847,7 +2866,7 @@
     </row>
     <row r="30" ht="19.5" customHeight="1">
       <c r="A30" t="s" s="14">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B30" s="15">
         <v>29</v>
@@ -2874,10 +2893,10 @@
     </row>
     <row r="31" ht="19.5" customHeight="1">
       <c r="A31" t="s" s="14">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B31" t="s" s="18">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C31" t="s" s="16">
         <v>17</v>
@@ -2901,7 +2920,7 @@
     </row>
     <row r="32" ht="19.5" customHeight="1">
       <c r="A32" t="s" s="14">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B32" s="15">
         <v>0</v>
@@ -2946,7 +2965,7 @@
     </row>
     <row r="33" ht="19.5" customHeight="1">
       <c r="A33" t="s" s="14">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B33" s="15">
         <v>0</v>

</xml_diff>

<commit_message>
add store byte opcode control
</commit_message>
<xml_diff>
--- a/scripts/mips32_r2000_instruction_set.xlsx
+++ b/scripts/mips32_r2000_instruction_set.xlsx
@@ -2358,16 +2358,36 @@
       <c r="E14" t="s" s="16">
         <v>17</v>
       </c>
-      <c r="F14" s="22"/>
-      <c r="G14" s="22"/>
-      <c r="H14" s="22"/>
-      <c r="I14" s="22"/>
-      <c r="J14" s="22"/>
-      <c r="K14" s="22"/>
-      <c r="L14" s="22"/>
-      <c r="M14" s="22"/>
-      <c r="N14" s="22"/>
-      <c r="O14" s="23"/>
+      <c r="F14" s="17">
+        <v>0</v>
+      </c>
+      <c r="G14" t="s" s="16">
+        <v>24</v>
+      </c>
+      <c r="H14" s="17">
+        <v>0</v>
+      </c>
+      <c r="I14" s="17">
+        <v>1</v>
+      </c>
+      <c r="J14" s="17">
+        <v>0</v>
+      </c>
+      <c r="K14" s="17">
+        <v>1</v>
+      </c>
+      <c r="L14" t="s" s="16">
+        <v>25</v>
+      </c>
+      <c r="M14" t="s" s="16">
+        <v>20</v>
+      </c>
+      <c r="N14" t="s" s="16">
+        <v>21</v>
+      </c>
+      <c r="O14" t="s" s="13">
+        <v>22</v>
+      </c>
     </row>
     <row r="15" ht="19.5" customHeight="1">
       <c r="A15" t="s" s="14">
@@ -2826,15 +2846,33 @@
       <c r="E28" t="s" s="16">
         <v>17</v>
       </c>
-      <c r="F28" s="22"/>
-      <c r="G28" s="22"/>
-      <c r="H28" s="22"/>
-      <c r="I28" s="22"/>
-      <c r="J28" s="22"/>
-      <c r="K28" s="22"/>
-      <c r="L28" s="22"/>
-      <c r="M28" s="22"/>
-      <c r="N28" s="22"/>
+      <c r="F28" s="19">
+        <v>0</v>
+      </c>
+      <c r="G28" s="19">
+        <v>0</v>
+      </c>
+      <c r="H28" s="19">
+        <v>0</v>
+      </c>
+      <c r="I28" s="19">
+        <v>0</v>
+      </c>
+      <c r="J28" s="19">
+        <v>1</v>
+      </c>
+      <c r="K28" s="19">
+        <v>0</v>
+      </c>
+      <c r="L28" t="s" s="16">
+        <v>25</v>
+      </c>
+      <c r="M28" t="s" s="16">
+        <v>20</v>
+      </c>
+      <c r="N28" t="s" s="16">
+        <v>21</v>
+      </c>
       <c r="O28" s="23"/>
     </row>
     <row r="29" ht="19.5" customHeight="1">
@@ -2907,16 +2945,36 @@
       <c r="E31" t="s" s="16">
         <v>17</v>
       </c>
-      <c r="F31" s="22"/>
-      <c r="G31" s="22"/>
-      <c r="H31" s="22"/>
-      <c r="I31" s="22"/>
-      <c r="J31" s="22"/>
-      <c r="K31" s="22"/>
-      <c r="L31" s="22"/>
-      <c r="M31" s="22"/>
-      <c r="N31" s="22"/>
-      <c r="O31" s="23"/>
+      <c r="F31" s="19">
+        <v>0</v>
+      </c>
+      <c r="G31" t="s" s="16">
+        <v>42</v>
+      </c>
+      <c r="H31" s="19">
+        <v>0</v>
+      </c>
+      <c r="I31" s="19">
+        <v>0</v>
+      </c>
+      <c r="J31" s="19">
+        <v>1</v>
+      </c>
+      <c r="K31" s="19">
+        <v>0</v>
+      </c>
+      <c r="L31" t="s" s="16">
+        <v>25</v>
+      </c>
+      <c r="M31" t="s" s="16">
+        <v>20</v>
+      </c>
+      <c r="N31" t="s" s="16">
+        <v>21</v>
+      </c>
+      <c r="O31" t="s" s="13">
+        <v>22</v>
+      </c>
     </row>
     <row r="32" ht="19.5" customHeight="1">
       <c r="A32" t="s" s="14">

</xml_diff>

<commit_message>
add sb and sh to control excel
</commit_message>
<xml_diff>
--- a/scripts/mips32_r2000_instruction_set.xlsx
+++ b/scripts/mips32_r2000_instruction_set.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="76">
   <si>
     <t>Table 1</t>
   </si>
@@ -220,10 +220,16 @@
     <t>sb</t>
   </si>
   <si>
+    <t>`SpecialOP_DM_BYTE</t>
+  </si>
+  <si>
     <t>sc</t>
   </si>
   <si>
     <t>sh</t>
+  </si>
+  <si>
+    <t>`SpecialOP_DM_HW</t>
   </si>
   <si>
     <t>sw</t>
@@ -2849,8 +2855,8 @@
       <c r="F28" s="19">
         <v>0</v>
       </c>
-      <c r="G28" s="19">
-        <v>0</v>
+      <c r="G28" t="s" s="16">
+        <v>42</v>
       </c>
       <c r="H28" s="19">
         <v>0</v>
@@ -2873,11 +2879,13 @@
       <c r="N28" t="s" s="16">
         <v>21</v>
       </c>
-      <c r="O28" s="23"/>
+      <c r="O28" t="s" s="13">
+        <v>69</v>
+      </c>
     </row>
     <row r="29" ht="19.5" customHeight="1">
       <c r="A29" t="s" s="14">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B29" s="15">
         <v>38</v>
@@ -2891,20 +2899,38 @@
       <c r="E29" t="s" s="16">
         <v>17</v>
       </c>
-      <c r="F29" s="22"/>
-      <c r="G29" s="22"/>
-      <c r="H29" s="22"/>
-      <c r="I29" s="22"/>
-      <c r="J29" s="22"/>
-      <c r="K29" s="22"/>
-      <c r="L29" s="22"/>
-      <c r="M29" s="22"/>
-      <c r="N29" s="22"/>
-      <c r="O29" s="23"/>
+      <c r="F29" s="19">
+        <v>0</v>
+      </c>
+      <c r="G29" t="s" s="16">
+        <v>42</v>
+      </c>
+      <c r="H29" s="19">
+        <v>0</v>
+      </c>
+      <c r="I29" s="19">
+        <v>0</v>
+      </c>
+      <c r="J29" s="19">
+        <v>1</v>
+      </c>
+      <c r="K29" s="19">
+        <v>0</v>
+      </c>
+      <c r="L29" t="s" s="16">
+        <v>25</v>
+      </c>
+      <c r="M29" t="s" s="16">
+        <v>20</v>
+      </c>
+      <c r="N29" t="s" s="16">
+        <v>21</v>
+      </c>
+      <c r="O29" s="13"/>
     </row>
     <row r="30" ht="19.5" customHeight="1">
       <c r="A30" t="s" s="14">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B30" s="15">
         <v>29</v>
@@ -2918,20 +2944,40 @@
       <c r="E30" t="s" s="16">
         <v>17</v>
       </c>
-      <c r="F30" s="22"/>
-      <c r="G30" s="22"/>
-      <c r="H30" s="22"/>
-      <c r="I30" s="22"/>
-      <c r="J30" s="22"/>
-      <c r="K30" s="22"/>
-      <c r="L30" s="22"/>
-      <c r="M30" s="22"/>
-      <c r="N30" s="22"/>
-      <c r="O30" s="23"/>
+      <c r="F30" s="19">
+        <v>0</v>
+      </c>
+      <c r="G30" t="s" s="16">
+        <v>42</v>
+      </c>
+      <c r="H30" s="19">
+        <v>0</v>
+      </c>
+      <c r="I30" s="19">
+        <v>0</v>
+      </c>
+      <c r="J30" s="19">
+        <v>1</v>
+      </c>
+      <c r="K30" s="19">
+        <v>0</v>
+      </c>
+      <c r="L30" t="s" s="16">
+        <v>25</v>
+      </c>
+      <c r="M30" t="s" s="16">
+        <v>20</v>
+      </c>
+      <c r="N30" t="s" s="16">
+        <v>21</v>
+      </c>
+      <c r="O30" t="s" s="13">
+        <v>72</v>
+      </c>
     </row>
     <row r="31" ht="19.5" customHeight="1">
       <c r="A31" t="s" s="14">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B31" t="s" s="18">
         <v>63</v>
@@ -2978,7 +3024,7 @@
     </row>
     <row r="32" ht="19.5" customHeight="1">
       <c r="A32" t="s" s="14">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B32" s="15">
         <v>0</v>
@@ -3023,7 +3069,7 @@
     </row>
     <row r="33" ht="19.5" customHeight="1">
       <c r="A33" t="s" s="14">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B33" s="15">
         <v>0</v>

</xml_diff>

<commit_message>
add load commands to control excel
</commit_message>
<xml_diff>
--- a/scripts/mips32_r2000_instruction_set.xlsx
+++ b/scripts/mips32_r2000_instruction_set.xlsx
@@ -148,9 +148,15 @@
     <t>lbu</t>
   </si>
   <si>
+    <t>`SpecialOP_DM_BYTE</t>
+  </si>
+  <si>
     <t>lhu</t>
   </si>
   <si>
+    <t>`SpecialOP_DM_HW</t>
+  </si>
+  <si>
     <t>ll</t>
   </si>
   <si>
@@ -220,16 +226,10 @@
     <t>sb</t>
   </si>
   <si>
-    <t>`SpecialOP_DM_BYTE</t>
-  </si>
-  <si>
     <t>sc</t>
   </si>
   <si>
     <t>sh</t>
-  </si>
-  <si>
-    <t>`SpecialOP_DM_HW</t>
   </si>
   <si>
     <t>sw</t>
@@ -2392,12 +2392,12 @@
         <v>21</v>
       </c>
       <c r="O14" t="s" s="13">
-        <v>22</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" ht="19.5" customHeight="1">
       <c r="A15" t="s" s="14">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B15" s="15">
         <v>25</v>
@@ -2411,20 +2411,40 @@
       <c r="E15" t="s" s="16">
         <v>17</v>
       </c>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="22"/>
-      <c r="I15" s="22"/>
-      <c r="J15" s="22"/>
-      <c r="K15" s="22"/>
-      <c r="L15" s="22"/>
-      <c r="M15" s="22"/>
-      <c r="N15" s="22"/>
-      <c r="O15" s="23"/>
+      <c r="F15" s="17">
+        <v>0</v>
+      </c>
+      <c r="G15" t="s" s="16">
+        <v>24</v>
+      </c>
+      <c r="H15" s="17">
+        <v>0</v>
+      </c>
+      <c r="I15" s="17">
+        <v>1</v>
+      </c>
+      <c r="J15" s="17">
+        <v>0</v>
+      </c>
+      <c r="K15" s="17">
+        <v>1</v>
+      </c>
+      <c r="L15" t="s" s="16">
+        <v>25</v>
+      </c>
+      <c r="M15" t="s" s="16">
+        <v>20</v>
+      </c>
+      <c r="N15" t="s" s="16">
+        <v>21</v>
+      </c>
+      <c r="O15" t="s" s="13">
+        <v>47</v>
+      </c>
     </row>
     <row r="16" ht="19.5" customHeight="1">
       <c r="A16" t="s" s="14">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B16" s="15">
         <v>30</v>
@@ -2438,23 +2458,43 @@
       <c r="E16" t="s" s="16">
         <v>17</v>
       </c>
-      <c r="F16" s="22"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="22"/>
-      <c r="I16" s="22"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="22"/>
-      <c r="L16" s="22"/>
-      <c r="M16" s="22"/>
-      <c r="N16" s="22"/>
-      <c r="O16" s="23"/>
+      <c r="F16" s="17">
+        <v>0</v>
+      </c>
+      <c r="G16" t="s" s="16">
+        <v>24</v>
+      </c>
+      <c r="H16" s="17">
+        <v>0</v>
+      </c>
+      <c r="I16" s="17">
+        <v>1</v>
+      </c>
+      <c r="J16" s="17">
+        <v>0</v>
+      </c>
+      <c r="K16" s="17">
+        <v>1</v>
+      </c>
+      <c r="L16" t="s" s="16">
+        <v>25</v>
+      </c>
+      <c r="M16" t="s" s="16">
+        <v>20</v>
+      </c>
+      <c r="N16" t="s" s="16">
+        <v>21</v>
+      </c>
+      <c r="O16" t="s" s="13">
+        <v>22</v>
+      </c>
     </row>
     <row r="17" ht="19.5" customHeight="1">
       <c r="A17" t="s" s="14">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B17" t="s" s="18">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C17" t="s" s="16">
         <v>17</v>
@@ -2478,7 +2518,7 @@
     </row>
     <row r="18" ht="19.5" customHeight="1">
       <c r="A18" t="s" s="14">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B18" s="15">
         <v>23</v>
@@ -2492,20 +2532,40 @@
       <c r="E18" t="s" s="16">
         <v>17</v>
       </c>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
-      <c r="J18" s="22"/>
-      <c r="K18" s="22"/>
-      <c r="L18" s="22"/>
-      <c r="M18" s="22"/>
-      <c r="N18" s="22"/>
-      <c r="O18" s="23"/>
+      <c r="F18" s="17">
+        <v>0</v>
+      </c>
+      <c r="G18" t="s" s="16">
+        <v>24</v>
+      </c>
+      <c r="H18" s="17">
+        <v>0</v>
+      </c>
+      <c r="I18" s="17">
+        <v>1</v>
+      </c>
+      <c r="J18" s="17">
+        <v>0</v>
+      </c>
+      <c r="K18" s="17">
+        <v>1</v>
+      </c>
+      <c r="L18" t="s" s="16">
+        <v>25</v>
+      </c>
+      <c r="M18" t="s" s="16">
+        <v>20</v>
+      </c>
+      <c r="N18" t="s" s="16">
+        <v>21</v>
+      </c>
+      <c r="O18" t="s" s="13">
+        <v>22</v>
+      </c>
     </row>
     <row r="19" ht="19.5" customHeight="1">
       <c r="A19" t="s" s="14">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B19" s="15">
         <v>0</v>
@@ -2544,13 +2604,13 @@
         <v>20</v>
       </c>
       <c r="N19" t="s" s="16">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="O19" s="13"/>
     </row>
     <row r="20" ht="19.5" customHeight="1">
       <c r="A20" t="s" s="14">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B20" s="15">
         <v>0</v>
@@ -2589,16 +2649,16 @@
         <v>20</v>
       </c>
       <c r="N20" t="s" s="16">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="O20" s="13"/>
     </row>
     <row r="21" ht="19.5" customHeight="1">
       <c r="A21" t="s" s="14">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B21" t="s" s="18">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C21" t="s" s="16">
         <v>17</v>
@@ -2634,13 +2694,13 @@
         <v>27</v>
       </c>
       <c r="N21" t="s" s="16">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="O21" s="13"/>
     </row>
     <row r="22" ht="19.5" customHeight="1">
       <c r="A22" t="s" s="14">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B22" s="15">
         <v>0</v>
@@ -2652,7 +2712,7 @@
         <v>17</v>
       </c>
       <c r="E22" t="s" s="16">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F22" s="22"/>
       <c r="G22" s="22"/>
@@ -2667,10 +2727,10 @@
     </row>
     <row r="23" ht="19.5" customHeight="1">
       <c r="A23" t="s" s="14">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B23" t="s" s="18">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C23" t="s" s="16">
         <v>17</v>
@@ -2694,10 +2754,10 @@
     </row>
     <row r="24" ht="19.5" customHeight="1">
       <c r="A24" t="s" s="14">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B24" t="s" s="18">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C24" t="s" s="16">
         <v>17</v>
@@ -2721,7 +2781,7 @@
     </row>
     <row r="25" ht="19.5" customHeight="1">
       <c r="A25" t="s" s="14">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B25" s="15">
         <v>0</v>
@@ -2733,7 +2793,7 @@
         <v>17</v>
       </c>
       <c r="E25" t="s" s="16">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F25" s="22"/>
       <c r="G25" s="22"/>
@@ -2748,7 +2808,7 @@
     </row>
     <row r="26" ht="19.5" customHeight="1">
       <c r="A26" t="s" s="14">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B26" s="15">
         <v>0</v>
@@ -2787,13 +2847,13 @@
         <v>20</v>
       </c>
       <c r="N26" t="s" s="16">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="O26" s="13"/>
     </row>
     <row r="27" ht="19.5" customHeight="1">
       <c r="A27" t="s" s="14">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B27" s="15">
         <v>0</v>
@@ -2832,13 +2892,13 @@
         <v>20</v>
       </c>
       <c r="N27" t="s" s="16">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O27" s="13"/>
     </row>
     <row r="28" ht="19.5" customHeight="1">
       <c r="A28" t="s" s="14">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B28" s="15">
         <v>28</v>
@@ -2880,12 +2940,12 @@
         <v>21</v>
       </c>
       <c r="O28" t="s" s="13">
-        <v>69</v>
+        <v>45</v>
       </c>
     </row>
     <row r="29" ht="19.5" customHeight="1">
       <c r="A29" t="s" s="14">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B29" s="15">
         <v>38</v>
@@ -2930,7 +2990,7 @@
     </row>
     <row r="30" ht="19.5" customHeight="1">
       <c r="A30" t="s" s="14">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B30" s="15">
         <v>29</v>
@@ -2972,7 +3032,7 @@
         <v>21</v>
       </c>
       <c r="O30" t="s" s="13">
-        <v>72</v>
+        <v>47</v>
       </c>
     </row>
     <row r="31" ht="19.5" customHeight="1">
@@ -2980,7 +3040,7 @@
         <v>73</v>
       </c>
       <c r="B31" t="s" s="18">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C31" t="s" s="16">
         <v>17</v>

</xml_diff>

<commit_message>
remove unsupported opcode from excel
</commit_message>
<xml_diff>
--- a/scripts/mips32_r2000_instruction_set.xlsx
+++ b/scripts/mips32_r2000_instruction_set.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="74">
   <si>
     <t>Table 1</t>
   </si>
@@ -157,9 +157,6 @@
     <t>`SpecialOP_DM_HW</t>
   </si>
   <si>
-    <t>ll</t>
-  </si>
-  <si>
     <t>lui</t>
   </si>
   <si>
@@ -224,9 +221,6 @@
   </si>
   <si>
     <t>sb</t>
-  </si>
-  <si>
-    <t>sc</t>
   </si>
   <si>
     <t>sh</t>
@@ -1758,7 +1752,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O70"/>
+  <dimension ref="A1:O68"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="15" width="16.3516" style="1" customWidth="1"/>
@@ -2446,8 +2440,8 @@
       <c r="A16" t="s" s="14">
         <v>48</v>
       </c>
-      <c r="B16" s="15">
-        <v>30</v>
+      <c r="B16" t="s" s="18">
+        <v>49</v>
       </c>
       <c r="C16" t="s" s="16">
         <v>17</v>
@@ -2458,44 +2452,24 @@
       <c r="E16" t="s" s="16">
         <v>17</v>
       </c>
-      <c r="F16" s="17">
-        <v>0</v>
-      </c>
-      <c r="G16" t="s" s="16">
-        <v>24</v>
-      </c>
-      <c r="H16" s="17">
-        <v>0</v>
-      </c>
-      <c r="I16" s="17">
-        <v>1</v>
-      </c>
-      <c r="J16" s="17">
-        <v>0</v>
-      </c>
-      <c r="K16" s="17">
-        <v>1</v>
-      </c>
-      <c r="L16" t="s" s="16">
-        <v>25</v>
-      </c>
-      <c r="M16" t="s" s="16">
-        <v>20</v>
-      </c>
-      <c r="N16" t="s" s="16">
-        <v>21</v>
-      </c>
-      <c r="O16" t="s" s="13">
-        <v>22</v>
-      </c>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="22"/>
+      <c r="J16" s="22"/>
+      <c r="K16" s="22"/>
+      <c r="L16" s="22"/>
+      <c r="M16" s="22"/>
+      <c r="N16" s="22"/>
+      <c r="O16" s="23"/>
     </row>
     <row r="17" ht="19.5" customHeight="1">
       <c r="A17" t="s" s="14">
-        <v>49</v>
-      </c>
-      <c r="B17" t="s" s="18">
         <v>50</v>
       </c>
+      <c r="B17" s="15">
+        <v>23</v>
+      </c>
       <c r="C17" t="s" s="16">
         <v>17</v>
       </c>
@@ -2505,23 +2479,43 @@
       <c r="E17" t="s" s="16">
         <v>17</v>
       </c>
-      <c r="F17" s="22"/>
-      <c r="G17" s="22"/>
-      <c r="H17" s="22"/>
-      <c r="I17" s="22"/>
-      <c r="J17" s="22"/>
-      <c r="K17" s="22"/>
-      <c r="L17" s="22"/>
-      <c r="M17" s="22"/>
-      <c r="N17" s="22"/>
-      <c r="O17" s="23"/>
+      <c r="F17" s="17">
+        <v>0</v>
+      </c>
+      <c r="G17" t="s" s="16">
+        <v>24</v>
+      </c>
+      <c r="H17" s="17">
+        <v>0</v>
+      </c>
+      <c r="I17" s="17">
+        <v>1</v>
+      </c>
+      <c r="J17" s="17">
+        <v>0</v>
+      </c>
+      <c r="K17" s="17">
+        <v>1</v>
+      </c>
+      <c r="L17" t="s" s="16">
+        <v>25</v>
+      </c>
+      <c r="M17" t="s" s="16">
+        <v>20</v>
+      </c>
+      <c r="N17" t="s" s="16">
+        <v>21</v>
+      </c>
+      <c r="O17" t="s" s="13">
+        <v>22</v>
+      </c>
     </row>
     <row r="18" ht="19.5" customHeight="1">
       <c r="A18" t="s" s="14">
         <v>51</v>
       </c>
       <c r="B18" s="15">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="C18" t="s" s="16">
         <v>17</v>
@@ -2529,20 +2523,20 @@
       <c r="D18" t="s" s="16">
         <v>17</v>
       </c>
-      <c r="E18" t="s" s="16">
-        <v>17</v>
+      <c r="E18" s="17">
+        <v>27</v>
       </c>
       <c r="F18" s="17">
         <v>0</v>
       </c>
       <c r="G18" t="s" s="16">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="H18" s="17">
         <v>0</v>
       </c>
       <c r="I18" s="17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18" s="17">
         <v>0</v>
@@ -2551,21 +2545,19 @@
         <v>1</v>
       </c>
       <c r="L18" t="s" s="16">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="M18" t="s" s="16">
         <v>20</v>
       </c>
       <c r="N18" t="s" s="16">
-        <v>21</v>
-      </c>
-      <c r="O18" t="s" s="13">
-        <v>22</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="O18" s="13"/>
     </row>
     <row r="19" ht="19.5" customHeight="1">
       <c r="A19" t="s" s="14">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B19" s="15">
         <v>0</v>
@@ -2577,7 +2569,7 @@
         <v>17</v>
       </c>
       <c r="E19" s="17">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F19" s="17">
         <v>0</v>
@@ -2604,16 +2596,16 @@
         <v>20</v>
       </c>
       <c r="N19" t="s" s="16">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="O19" s="13"/>
     </row>
     <row r="20" ht="19.5" customHeight="1">
       <c r="A20" t="s" s="14">
-        <v>54</v>
-      </c>
-      <c r="B20" s="15">
-        <v>0</v>
+        <v>55</v>
+      </c>
+      <c r="B20" t="s" s="18">
+        <v>56</v>
       </c>
       <c r="C20" t="s" s="16">
         <v>17</v>
@@ -2621,14 +2613,14 @@
       <c r="D20" t="s" s="16">
         <v>17</v>
       </c>
-      <c r="E20" s="17">
-        <v>25</v>
+      <c r="E20" t="s" s="16">
+        <v>17</v>
       </c>
       <c r="F20" s="17">
         <v>0</v>
       </c>
       <c r="G20" t="s" s="16">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="H20" s="17">
         <v>0</v>
@@ -2643,23 +2635,23 @@
         <v>1</v>
       </c>
       <c r="L20" t="s" s="16">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="M20" t="s" s="16">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="N20" t="s" s="16">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O20" s="13"/>
     </row>
     <row r="21" ht="19.5" customHeight="1">
       <c r="A21" t="s" s="14">
-        <v>56</v>
-      </c>
-      <c r="B21" t="s" s="18">
         <v>57</v>
       </c>
+      <c r="B21" s="15">
+        <v>0</v>
+      </c>
       <c r="C21" t="s" s="16">
         <v>17</v>
       </c>
@@ -2667,43 +2659,25 @@
         <v>17</v>
       </c>
       <c r="E21" t="s" s="16">
-        <v>17</v>
-      </c>
-      <c r="F21" s="17">
-        <v>0</v>
-      </c>
-      <c r="G21" t="s" s="16">
-        <v>24</v>
-      </c>
-      <c r="H21" s="17">
-        <v>0</v>
-      </c>
-      <c r="I21" s="17">
-        <v>0</v>
-      </c>
-      <c r="J21" s="17">
-        <v>0</v>
-      </c>
-      <c r="K21" s="17">
-        <v>1</v>
-      </c>
-      <c r="L21" t="s" s="16">
-        <v>25</v>
-      </c>
-      <c r="M21" t="s" s="16">
-        <v>27</v>
-      </c>
-      <c r="N21" t="s" s="16">
-        <v>55</v>
-      </c>
-      <c r="O21" s="13"/>
+        <v>58</v>
+      </c>
+      <c r="F21" s="22"/>
+      <c r="G21" s="22"/>
+      <c r="H21" s="22"/>
+      <c r="I21" s="22"/>
+      <c r="J21" s="22"/>
+      <c r="K21" s="22"/>
+      <c r="L21" s="22"/>
+      <c r="M21" s="22"/>
+      <c r="N21" s="22"/>
+      <c r="O21" s="23"/>
     </row>
     <row r="22" ht="19.5" customHeight="1">
       <c r="A22" t="s" s="14">
-        <v>58</v>
-      </c>
-      <c r="B22" s="15">
-        <v>0</v>
+        <v>59</v>
+      </c>
+      <c r="B22" t="s" s="18">
+        <v>60</v>
       </c>
       <c r="C22" t="s" s="16">
         <v>17</v>
@@ -2712,7 +2686,7 @@
         <v>17</v>
       </c>
       <c r="E22" t="s" s="16">
-        <v>59</v>
+        <v>17</v>
       </c>
       <c r="F22" s="22"/>
       <c r="G22" s="22"/>
@@ -2727,10 +2701,10 @@
     </row>
     <row r="23" ht="19.5" customHeight="1">
       <c r="A23" t="s" s="14">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B23" t="s" s="18">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C23" t="s" s="16">
         <v>17</v>
@@ -2754,11 +2728,11 @@
     </row>
     <row r="24" ht="19.5" customHeight="1">
       <c r="A24" t="s" s="14">
-        <v>62</v>
-      </c>
-      <c r="B24" t="s" s="18">
         <v>63</v>
       </c>
+      <c r="B24" s="15">
+        <v>0</v>
+      </c>
       <c r="C24" t="s" s="16">
         <v>17</v>
       </c>
@@ -2766,7 +2740,7 @@
         <v>17</v>
       </c>
       <c r="E24" t="s" s="16">
-        <v>17</v>
+        <v>64</v>
       </c>
       <c r="F24" s="22"/>
       <c r="G24" s="22"/>
@@ -2781,7 +2755,7 @@
     </row>
     <row r="25" ht="19.5" customHeight="1">
       <c r="A25" t="s" s="14">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B25" s="15">
         <v>0</v>
@@ -2792,23 +2766,41 @@
       <c r="D25" t="s" s="16">
         <v>17</v>
       </c>
-      <c r="E25" t="s" s="16">
-        <v>65</v>
-      </c>
-      <c r="F25" s="22"/>
-      <c r="G25" s="22"/>
-      <c r="H25" s="22"/>
-      <c r="I25" s="22"/>
-      <c r="J25" s="22"/>
-      <c r="K25" s="22"/>
-      <c r="L25" s="22"/>
-      <c r="M25" s="22"/>
-      <c r="N25" s="22"/>
-      <c r="O25" s="23"/>
+      <c r="E25" s="17">
+        <v>0</v>
+      </c>
+      <c r="F25" s="17">
+        <v>0</v>
+      </c>
+      <c r="G25" t="s" s="16">
+        <v>18</v>
+      </c>
+      <c r="H25" s="17">
+        <v>0</v>
+      </c>
+      <c r="I25" s="17">
+        <v>0</v>
+      </c>
+      <c r="J25" s="17">
+        <v>0</v>
+      </c>
+      <c r="K25" s="17">
+        <v>1</v>
+      </c>
+      <c r="L25" t="s" s="16">
+        <v>19</v>
+      </c>
+      <c r="M25" t="s" s="16">
+        <v>20</v>
+      </c>
+      <c r="N25" t="s" s="16">
+        <v>66</v>
+      </c>
+      <c r="O25" s="13"/>
     </row>
     <row r="26" ht="19.5" customHeight="1">
       <c r="A26" t="s" s="14">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B26" s="15">
         <v>0</v>
@@ -2820,7 +2812,7 @@
         <v>17</v>
       </c>
       <c r="E26" s="17">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F26" s="17">
         <v>0</v>
@@ -2847,16 +2839,16 @@
         <v>20</v>
       </c>
       <c r="N26" t="s" s="16">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="O26" s="13"/>
     </row>
     <row r="27" ht="19.5" customHeight="1">
       <c r="A27" t="s" s="14">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B27" s="15">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="C27" t="s" s="16">
         <v>17</v>
@@ -2864,44 +2856,46 @@
       <c r="D27" t="s" s="16">
         <v>17</v>
       </c>
-      <c r="E27" s="17">
-        <v>2</v>
-      </c>
-      <c r="F27" s="17">
+      <c r="E27" t="s" s="16">
+        <v>17</v>
+      </c>
+      <c r="F27" s="19">
         <v>0</v>
       </c>
       <c r="G27" t="s" s="16">
-        <v>18</v>
-      </c>
-      <c r="H27" s="17">
-        <v>0</v>
-      </c>
-      <c r="I27" s="17">
-        <v>0</v>
-      </c>
-      <c r="J27" s="17">
-        <v>0</v>
-      </c>
-      <c r="K27" s="17">
+        <v>42</v>
+      </c>
+      <c r="H27" s="19">
+        <v>0</v>
+      </c>
+      <c r="I27" s="19">
+        <v>0</v>
+      </c>
+      <c r="J27" s="19">
         <v>1</v>
       </c>
+      <c r="K27" s="19">
+        <v>0</v>
+      </c>
       <c r="L27" t="s" s="16">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="M27" t="s" s="16">
         <v>20</v>
       </c>
       <c r="N27" t="s" s="16">
-        <v>69</v>
-      </c>
-      <c r="O27" s="13"/>
+        <v>21</v>
+      </c>
+      <c r="O27" t="s" s="13">
+        <v>45</v>
+      </c>
     </row>
     <row r="28" ht="19.5" customHeight="1">
       <c r="A28" t="s" s="14">
         <v>70</v>
       </c>
       <c r="B28" s="15">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C28" t="s" s="16">
         <v>17</v>
@@ -2940,15 +2934,15 @@
         <v>21</v>
       </c>
       <c r="O28" t="s" s="13">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="29" ht="19.5" customHeight="1">
       <c r="A29" t="s" s="14">
         <v>71</v>
       </c>
-      <c r="B29" s="15">
-        <v>38</v>
+      <c r="B29" t="s" s="18">
+        <v>64</v>
       </c>
       <c r="C29" t="s" s="16">
         <v>17</v>
@@ -2986,14 +2980,16 @@
       <c r="N29" t="s" s="16">
         <v>21</v>
       </c>
-      <c r="O29" s="13"/>
+      <c r="O29" t="s" s="13">
+        <v>22</v>
+      </c>
     </row>
     <row r="30" ht="19.5" customHeight="1">
       <c r="A30" t="s" s="14">
         <v>72</v>
       </c>
       <c r="B30" s="15">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="C30" t="s" s="16">
         <v>17</v>
@@ -3001,46 +2997,44 @@
       <c r="D30" t="s" s="16">
         <v>17</v>
       </c>
-      <c r="E30" t="s" s="16">
-        <v>17</v>
-      </c>
-      <c r="F30" s="19">
+      <c r="E30" s="17">
+        <v>22</v>
+      </c>
+      <c r="F30" s="17">
         <v>0</v>
       </c>
       <c r="G30" t="s" s="16">
-        <v>42</v>
-      </c>
-      <c r="H30" s="19">
-        <v>0</v>
-      </c>
-      <c r="I30" s="19">
-        <v>0</v>
-      </c>
-      <c r="J30" s="19">
+        <v>18</v>
+      </c>
+      <c r="H30" s="17">
+        <v>0</v>
+      </c>
+      <c r="I30" s="17">
+        <v>0</v>
+      </c>
+      <c r="J30" s="17">
+        <v>0</v>
+      </c>
+      <c r="K30" s="17">
         <v>1</v>
       </c>
-      <c r="K30" s="19">
-        <v>0</v>
-      </c>
       <c r="L30" t="s" s="16">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="M30" t="s" s="16">
         <v>20</v>
       </c>
       <c r="N30" t="s" s="16">
-        <v>21</v>
-      </c>
-      <c r="O30" t="s" s="13">
-        <v>47</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="O30" s="13"/>
     </row>
     <row r="31" ht="19.5" customHeight="1">
       <c r="A31" t="s" s="14">
         <v>73</v>
       </c>
-      <c r="B31" t="s" s="18">
-        <v>65</v>
+      <c r="B31" s="15">
+        <v>0</v>
       </c>
       <c r="C31" t="s" s="16">
         <v>17</v>
@@ -3048,129 +3042,71 @@
       <c r="D31" t="s" s="16">
         <v>17</v>
       </c>
-      <c r="E31" t="s" s="16">
-        <v>17</v>
-      </c>
-      <c r="F31" s="19">
+      <c r="E31" s="17">
+        <v>23</v>
+      </c>
+      <c r="F31" s="17">
         <v>0</v>
       </c>
       <c r="G31" t="s" s="16">
-        <v>42</v>
-      </c>
-      <c r="H31" s="19">
-        <v>0</v>
-      </c>
-      <c r="I31" s="19">
-        <v>0</v>
-      </c>
-      <c r="J31" s="19">
+        <v>18</v>
+      </c>
+      <c r="H31" s="17">
+        <v>0</v>
+      </c>
+      <c r="I31" s="17">
+        <v>0</v>
+      </c>
+      <c r="J31" s="17">
+        <v>0</v>
+      </c>
+      <c r="K31" s="17">
         <v>1</v>
       </c>
-      <c r="K31" s="19">
-        <v>0</v>
-      </c>
       <c r="L31" t="s" s="16">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="M31" t="s" s="16">
         <v>20</v>
       </c>
       <c r="N31" t="s" s="16">
-        <v>21</v>
-      </c>
-      <c r="O31" t="s" s="13">
-        <v>22</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="O31" s="13"/>
     </row>
     <row r="32" ht="19.5" customHeight="1">
-      <c r="A32" t="s" s="14">
-        <v>74</v>
-      </c>
-      <c r="B32" s="15">
-        <v>0</v>
-      </c>
-      <c r="C32" t="s" s="16">
-        <v>17</v>
-      </c>
-      <c r="D32" t="s" s="16">
-        <v>17</v>
-      </c>
-      <c r="E32" s="17">
-        <v>22</v>
-      </c>
-      <c r="F32" s="17">
-        <v>0</v>
-      </c>
-      <c r="G32" t="s" s="16">
-        <v>18</v>
-      </c>
-      <c r="H32" s="17">
-        <v>0</v>
-      </c>
-      <c r="I32" s="17">
-        <v>0</v>
-      </c>
-      <c r="J32" s="17">
-        <v>0</v>
-      </c>
-      <c r="K32" s="17">
-        <v>1</v>
-      </c>
-      <c r="L32" t="s" s="16">
-        <v>19</v>
-      </c>
-      <c r="M32" t="s" s="16">
-        <v>20</v>
-      </c>
-      <c r="N32" t="s" s="16">
-        <v>34</v>
-      </c>
-      <c r="O32" s="13"/>
+      <c r="A32" s="24"/>
+      <c r="B32" s="25"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="I32" s="22"/>
+      <c r="J32" s="22"/>
+      <c r="K32" s="22"/>
+      <c r="L32" s="22"/>
+      <c r="M32" s="22"/>
+      <c r="N32" s="22"/>
+      <c r="O32" s="23"/>
     </row>
     <row r="33" ht="19.5" customHeight="1">
-      <c r="A33" t="s" s="14">
-        <v>75</v>
-      </c>
-      <c r="B33" s="15">
-        <v>0</v>
-      </c>
-      <c r="C33" t="s" s="16">
-        <v>17</v>
-      </c>
-      <c r="D33" t="s" s="16">
-        <v>17</v>
-      </c>
-      <c r="E33" s="17">
-        <v>23</v>
-      </c>
-      <c r="F33" s="17">
-        <v>0</v>
-      </c>
-      <c r="G33" t="s" s="16">
-        <v>18</v>
-      </c>
-      <c r="H33" s="17">
-        <v>0</v>
-      </c>
-      <c r="I33" s="17">
-        <v>0</v>
-      </c>
-      <c r="J33" s="17">
-        <v>0</v>
-      </c>
-      <c r="K33" s="17">
-        <v>1</v>
-      </c>
-      <c r="L33" t="s" s="16">
-        <v>19</v>
-      </c>
-      <c r="M33" t="s" s="16">
-        <v>20</v>
-      </c>
-      <c r="N33" t="s" s="16">
-        <v>34</v>
-      </c>
-      <c r="O33" s="13"/>
+      <c r="A33" s="24"/>
+      <c r="B33" s="25"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="22"/>
+      <c r="E33" s="22"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="22"/>
+      <c r="H33" s="22"/>
+      <c r="I33" s="22"/>
+      <c r="J33" s="22"/>
+      <c r="K33" s="22"/>
+      <c r="L33" s="22"/>
+      <c r="M33" s="22"/>
+      <c r="N33" s="22"/>
+      <c r="O33" s="23"/>
     </row>
     <row r="34" ht="19.5" customHeight="1">
       <c r="A34" s="24"/>
@@ -3751,55 +3687,21 @@
       <c r="O67" s="23"/>
     </row>
     <row r="68" ht="19.5" customHeight="1">
-      <c r="A68" s="24"/>
-      <c r="B68" s="25"/>
-      <c r="C68" s="22"/>
-      <c r="D68" s="22"/>
-      <c r="E68" s="22"/>
-      <c r="F68" s="22"/>
-      <c r="G68" s="22"/>
-      <c r="H68" s="22"/>
-      <c r="I68" s="22"/>
-      <c r="J68" s="22"/>
-      <c r="K68" s="22"/>
-      <c r="L68" s="22"/>
-      <c r="M68" s="22"/>
-      <c r="N68" s="22"/>
-      <c r="O68" s="23"/>
-    </row>
-    <row r="69" ht="19.5" customHeight="1">
-      <c r="A69" s="24"/>
-      <c r="B69" s="25"/>
-      <c r="C69" s="22"/>
-      <c r="D69" s="22"/>
-      <c r="E69" s="22"/>
-      <c r="F69" s="22"/>
-      <c r="G69" s="22"/>
-      <c r="H69" s="22"/>
-      <c r="I69" s="22"/>
-      <c r="J69" s="22"/>
-      <c r="K69" s="22"/>
-      <c r="L69" s="22"/>
-      <c r="M69" s="22"/>
-      <c r="N69" s="22"/>
-      <c r="O69" s="23"/>
-    </row>
-    <row r="70" ht="19.5" customHeight="1">
-      <c r="A70" s="26"/>
-      <c r="B70" s="27"/>
-      <c r="C70" s="28"/>
-      <c r="D70" s="28"/>
-      <c r="E70" s="28"/>
-      <c r="F70" s="28"/>
-      <c r="G70" s="28"/>
-      <c r="H70" s="28"/>
-      <c r="I70" s="28"/>
-      <c r="J70" s="28"/>
-      <c r="K70" s="28"/>
-      <c r="L70" s="28"/>
-      <c r="M70" s="28"/>
-      <c r="N70" s="28"/>
-      <c r="O70" s="29"/>
+      <c r="A68" s="26"/>
+      <c r="B68" s="27"/>
+      <c r="C68" s="28"/>
+      <c r="D68" s="28"/>
+      <c r="E68" s="28"/>
+      <c r="F68" s="28"/>
+      <c r="G68" s="28"/>
+      <c r="H68" s="28"/>
+      <c r="I68" s="28"/>
+      <c r="J68" s="28"/>
+      <c r="K68" s="28"/>
+      <c r="L68" s="28"/>
+      <c r="M68" s="28"/>
+      <c r="N68" s="28"/>
+      <c r="O68" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
add lui to control excel
</commit_message>
<xml_diff>
--- a/scripts/mips32_r2000_instruction_set.xlsx
+++ b/scripts/mips32_r2000_instruction_set.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="75">
   <si>
     <t>Table 1</t>
   </si>
@@ -161,6 +161,9 @@
   </si>
   <si>
     <t>f</t>
+  </si>
+  <si>
+    <t>`ALUOp_LUI</t>
   </si>
   <si>
     <t>lw</t>
@@ -2452,20 +2455,40 @@
       <c r="E16" t="s" s="16">
         <v>17</v>
       </c>
-      <c r="F16" s="22"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="22"/>
-      <c r="I16" s="22"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="22"/>
-      <c r="L16" s="22"/>
-      <c r="M16" s="22"/>
-      <c r="N16" s="22"/>
-      <c r="O16" s="23"/>
+      <c r="F16" s="17">
+        <v>0</v>
+      </c>
+      <c r="G16" t="s" s="16">
+        <v>24</v>
+      </c>
+      <c r="H16" s="17">
+        <v>0</v>
+      </c>
+      <c r="I16" s="17">
+        <v>0</v>
+      </c>
+      <c r="J16" s="17">
+        <v>0</v>
+      </c>
+      <c r="K16" s="17">
+        <v>0</v>
+      </c>
+      <c r="L16" t="s" s="16">
+        <v>25</v>
+      </c>
+      <c r="M16" t="s" s="16">
+        <v>27</v>
+      </c>
+      <c r="N16" t="s" s="16">
+        <v>50</v>
+      </c>
+      <c r="O16" t="s" s="13">
+        <v>22</v>
+      </c>
     </row>
     <row r="17" ht="19.5" customHeight="1">
       <c r="A17" t="s" s="14">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B17" s="15">
         <v>23</v>
@@ -2512,7 +2535,7 @@
     </row>
     <row r="18" ht="19.5" customHeight="1">
       <c r="A18" t="s" s="14">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B18" s="15">
         <v>0</v>
@@ -2551,13 +2574,13 @@
         <v>20</v>
       </c>
       <c r="N18" t="s" s="16">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="O18" s="13"/>
     </row>
     <row r="19" ht="19.5" customHeight="1">
       <c r="A19" t="s" s="14">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B19" s="15">
         <v>0</v>
@@ -2596,16 +2619,16 @@
         <v>20</v>
       </c>
       <c r="N19" t="s" s="16">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O19" s="13"/>
     </row>
     <row r="20" ht="19.5" customHeight="1">
       <c r="A20" t="s" s="14">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B20" t="s" s="18">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C20" t="s" s="16">
         <v>17</v>
@@ -2641,13 +2664,13 @@
         <v>27</v>
       </c>
       <c r="N20" t="s" s="16">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O20" s="13"/>
     </row>
     <row r="21" ht="19.5" customHeight="1">
       <c r="A21" t="s" s="14">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B21" s="15">
         <v>0</v>
@@ -2659,7 +2682,7 @@
         <v>17</v>
       </c>
       <c r="E21" t="s" s="16">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F21" s="22"/>
       <c r="G21" s="22"/>
@@ -2674,10 +2697,10 @@
     </row>
     <row r="22" ht="19.5" customHeight="1">
       <c r="A22" t="s" s="14">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B22" t="s" s="18">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C22" t="s" s="16">
         <v>17</v>
@@ -2701,10 +2724,10 @@
     </row>
     <row r="23" ht="19.5" customHeight="1">
       <c r="A23" t="s" s="14">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B23" t="s" s="18">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C23" t="s" s="16">
         <v>17</v>
@@ -2728,7 +2751,7 @@
     </row>
     <row r="24" ht="19.5" customHeight="1">
       <c r="A24" t="s" s="14">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B24" s="15">
         <v>0</v>
@@ -2740,7 +2763,7 @@
         <v>17</v>
       </c>
       <c r="E24" t="s" s="16">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F24" s="22"/>
       <c r="G24" s="22"/>
@@ -2755,7 +2778,7 @@
     </row>
     <row r="25" ht="19.5" customHeight="1">
       <c r="A25" t="s" s="14">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B25" s="15">
         <v>0</v>
@@ -2794,13 +2817,13 @@
         <v>20</v>
       </c>
       <c r="N25" t="s" s="16">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="O25" s="13"/>
     </row>
     <row r="26" ht="19.5" customHeight="1">
       <c r="A26" t="s" s="14">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B26" s="15">
         <v>0</v>
@@ -2839,13 +2862,13 @@
         <v>20</v>
       </c>
       <c r="N26" t="s" s="16">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="O26" s="13"/>
     </row>
     <row r="27" ht="19.5" customHeight="1">
       <c r="A27" t="s" s="14">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B27" s="15">
         <v>28</v>
@@ -2892,7 +2915,7 @@
     </row>
     <row r="28" ht="19.5" customHeight="1">
       <c r="A28" t="s" s="14">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B28" s="15">
         <v>29</v>
@@ -2939,10 +2962,10 @@
     </row>
     <row r="29" ht="19.5" customHeight="1">
       <c r="A29" t="s" s="14">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B29" t="s" s="18">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C29" t="s" s="16">
         <v>17</v>
@@ -2986,7 +3009,7 @@
     </row>
     <row r="30" ht="19.5" customHeight="1">
       <c r="A30" t="s" s="14">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B30" s="15">
         <v>0</v>
@@ -3031,7 +3054,7 @@
     </row>
     <row r="31" ht="19.5" customHeight="1">
       <c r="A31" t="s" s="14">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B31" s="15">
         <v>0</v>

</xml_diff>

<commit_message>
add lb opcode to control
</commit_message>
<xml_diff>
--- a/scripts/mips32_r2000_instruction_set.xlsx
+++ b/scripts/mips32_r2000_instruction_set.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="77">
   <si>
     <t>Table 1</t>
   </si>
@@ -239,6 +239,9 @@
   </si>
   <si>
     <t>subu</t>
+  </si>
+  <si>
+    <t>lb</t>
   </si>
 </sst>
 </file>
@@ -3195,21 +3198,51 @@
       </c>
     </row>
     <row r="32" ht="19.5" customHeight="1">
-      <c r="A32" s="22"/>
-      <c r="B32" s="23"/>
-      <c r="C32" s="24"/>
-      <c r="D32" s="24"/>
-      <c r="E32" s="24"/>
-      <c r="F32" s="24"/>
-      <c r="G32" s="24"/>
-      <c r="H32" s="24"/>
-      <c r="I32" s="24"/>
-      <c r="J32" s="24"/>
-      <c r="K32" s="24"/>
-      <c r="L32" s="24"/>
-      <c r="M32" s="24"/>
-      <c r="N32" s="24"/>
-      <c r="O32" s="25"/>
+      <c r="A32" t="s" s="14">
+        <v>76</v>
+      </c>
+      <c r="B32" s="15">
+        <v>20</v>
+      </c>
+      <c r="C32" t="s" s="16">
+        <v>17</v>
+      </c>
+      <c r="D32" t="s" s="16">
+        <v>17</v>
+      </c>
+      <c r="E32" t="s" s="16">
+        <v>17</v>
+      </c>
+      <c r="F32" s="17">
+        <v>0</v>
+      </c>
+      <c r="G32" t="s" s="16">
+        <v>24</v>
+      </c>
+      <c r="H32" s="17">
+        <v>0</v>
+      </c>
+      <c r="I32" s="17">
+        <v>1</v>
+      </c>
+      <c r="J32" s="17">
+        <v>0</v>
+      </c>
+      <c r="K32" s="17">
+        <v>1</v>
+      </c>
+      <c r="L32" t="s" s="16">
+        <v>25</v>
+      </c>
+      <c r="M32" t="s" s="16">
+        <v>20</v>
+      </c>
+      <c r="N32" t="s" s="16">
+        <v>21</v>
+      </c>
+      <c r="O32" t="s" s="13">
+        <v>45</v>
+      </c>
     </row>
     <row r="33" ht="19.5" customHeight="1">
       <c r="A33" s="22"/>

</xml_diff>

<commit_message>
add bgtz and blez instructions to control
</commit_message>
<xml_diff>
--- a/scripts/mips32_r2000_instruction_set.xlsx
+++ b/scripts/mips32_r2000_instruction_set.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="85">
   <si>
     <t>Table 1</t>
   </si>
@@ -118,10 +118,13 @@
     <t>`ALUOp_SUB</t>
   </si>
   <si>
+    <t>`SpecialOP_BEQ</t>
+  </si>
+  <si>
     <t>bne</t>
   </si>
   <si>
-    <t>`ALUOp_BNE</t>
+    <t>`SpecialOP_BNE</t>
   </si>
   <si>
     <t>j</t>
@@ -251,6 +254,18 @@
   </si>
   <si>
     <t>nop</t>
+  </si>
+  <si>
+    <t>bgtz</t>
+  </si>
+  <si>
+    <t>`SpecialOP_BGTZ</t>
+  </si>
+  <si>
+    <t>blez</t>
+  </si>
+  <si>
+    <t>`SpecialOP_BLEZ</t>
   </si>
 </sst>
 </file>
@@ -625,7 +640,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -702,6 +717,9 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="14" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -2172,12 +2190,12 @@
         <v>34</v>
       </c>
       <c r="O9" t="s" s="13">
-        <v>22</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" ht="19.5" customHeight="1">
       <c r="A10" t="s" s="14">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B10" s="15">
         <v>5</v>
@@ -2216,15 +2234,15 @@
         <v>20</v>
       </c>
       <c r="N10" t="s" s="16">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="O10" t="s" s="13">
-        <v>22</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" ht="19.5" customHeight="1">
       <c r="A11" t="s" s="14">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B11" s="15">
         <v>2</v>
@@ -2271,7 +2289,7 @@
     </row>
     <row r="12" ht="19.5" customHeight="1">
       <c r="A12" t="s" s="14">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B12" s="15">
         <v>3</v>
@@ -2310,15 +2328,15 @@
         <v>0</v>
       </c>
       <c r="N12" t="s" s="21">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="O12" t="s" s="13">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" ht="19.5" customHeight="1">
       <c r="A13" t="s" s="14">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B13" s="15">
         <v>0</v>
@@ -2336,7 +2354,7 @@
         <v>1</v>
       </c>
       <c r="G13" t="s" s="16">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H13" s="17">
         <v>0</v>
@@ -2357,15 +2375,15 @@
         <v>0</v>
       </c>
       <c r="N13" t="s" s="11">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="O13" t="s" s="13">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" ht="19.5" customHeight="1">
       <c r="A14" t="s" s="14">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B14" s="15">
         <v>24</v>
@@ -2407,12 +2425,12 @@
         <v>21</v>
       </c>
       <c r="O14" t="s" s="13">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" ht="19.5" customHeight="1">
       <c r="A15" t="s" s="14">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B15" s="15">
         <v>25</v>
@@ -2454,15 +2472,15 @@
         <v>21</v>
       </c>
       <c r="O15" t="s" s="13">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" ht="19.5" customHeight="1">
       <c r="A16" t="s" s="14">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B16" t="s" s="18">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C16" t="s" s="16">
         <v>17</v>
@@ -2498,7 +2516,7 @@
         <v>27</v>
       </c>
       <c r="N16" t="s" s="16">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="O16" t="s" s="13">
         <v>22</v>
@@ -2506,7 +2524,7 @@
     </row>
     <row r="17" ht="19.5" customHeight="1">
       <c r="A17" t="s" s="14">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B17" s="15">
         <v>23</v>
@@ -2553,7 +2571,7 @@
     </row>
     <row r="18" ht="19.5" customHeight="1">
       <c r="A18" t="s" s="14">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B18" s="15">
         <v>0</v>
@@ -2592,7 +2610,7 @@
         <v>20</v>
       </c>
       <c r="N18" t="s" s="16">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="O18" t="s" s="13">
         <v>22</v>
@@ -2600,7 +2618,7 @@
     </row>
     <row r="19" ht="19.5" customHeight="1">
       <c r="A19" t="s" s="14">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B19" s="15">
         <v>0</v>
@@ -2639,7 +2657,7 @@
         <v>20</v>
       </c>
       <c r="N19" t="s" s="16">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="O19" t="s" s="13">
         <v>22</v>
@@ -2647,10 +2665,10 @@
     </row>
     <row r="20" ht="19.5" customHeight="1">
       <c r="A20" t="s" s="14">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B20" t="s" s="18">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C20" t="s" s="16">
         <v>17</v>
@@ -2686,7 +2704,7 @@
         <v>27</v>
       </c>
       <c r="N20" t="s" s="16">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="O20" t="s" s="13">
         <v>22</v>
@@ -2694,7 +2712,7 @@
     </row>
     <row r="21" ht="19.5" customHeight="1">
       <c r="A21" t="s" s="14">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B21" s="15">
         <v>0</v>
@@ -2706,7 +2724,7 @@
         <v>17</v>
       </c>
       <c r="E21" t="s" s="16">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F21" s="17">
         <v>0</v>
@@ -2733,7 +2751,7 @@
         <v>20</v>
       </c>
       <c r="N21" t="s" s="16">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="O21" t="s" s="13">
         <v>22</v>
@@ -2741,10 +2759,10 @@
     </row>
     <row r="22" ht="19.5" customHeight="1">
       <c r="A22" t="s" s="14">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B22" t="s" s="18">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C22" t="s" s="16">
         <v>17</v>
@@ -2780,7 +2798,7 @@
         <v>20</v>
       </c>
       <c r="N22" t="s" s="16">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="O22" t="s" s="13">
         <v>22</v>
@@ -2788,10 +2806,10 @@
     </row>
     <row r="23" ht="19.5" customHeight="1">
       <c r="A23" t="s" s="14">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B23" t="s" s="18">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C23" t="s" s="16">
         <v>17</v>
@@ -2827,7 +2845,7 @@
         <v>27</v>
       </c>
       <c r="N23" t="s" s="16">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="O23" t="s" s="13">
         <v>22</v>
@@ -2835,7 +2853,7 @@
     </row>
     <row r="24" ht="19.5" customHeight="1">
       <c r="A24" t="s" s="14">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B24" s="15">
         <v>0</v>
@@ -2847,7 +2865,7 @@
         <v>17</v>
       </c>
       <c r="E24" t="s" s="16">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F24" s="17">
         <v>0</v>
@@ -2874,7 +2892,7 @@
         <v>27</v>
       </c>
       <c r="N24" t="s" s="16">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="O24" t="s" s="13">
         <v>22</v>
@@ -2882,7 +2900,7 @@
     </row>
     <row r="25" ht="19.5" customHeight="1">
       <c r="A25" t="s" s="14">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B25" s="15">
         <v>0</v>
@@ -2921,7 +2939,7 @@
         <v>20</v>
       </c>
       <c r="N25" t="s" s="16">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="O25" t="s" s="13">
         <v>22</v>
@@ -2929,7 +2947,7 @@
     </row>
     <row r="26" ht="19.5" customHeight="1">
       <c r="A26" t="s" s="14">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B26" s="15">
         <v>0</v>
@@ -2968,7 +2986,7 @@
         <v>20</v>
       </c>
       <c r="N26" t="s" s="16">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O26" t="s" s="13">
         <v>22</v>
@@ -2976,7 +2994,7 @@
     </row>
     <row r="27" ht="19.5" customHeight="1">
       <c r="A27" t="s" s="14">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B27" s="15">
         <v>28</v>
@@ -2994,7 +3012,7 @@
         <v>0</v>
       </c>
       <c r="G27" t="s" s="16">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H27" s="19">
         <v>0</v>
@@ -3018,12 +3036,12 @@
         <v>21</v>
       </c>
       <c r="O27" t="s" s="13">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="28" ht="19.5" customHeight="1">
       <c r="A28" t="s" s="14">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B28" s="15">
         <v>29</v>
@@ -3041,7 +3059,7 @@
         <v>0</v>
       </c>
       <c r="G28" t="s" s="16">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H28" s="19">
         <v>0</v>
@@ -3065,15 +3083,15 @@
         <v>21</v>
       </c>
       <c r="O28" t="s" s="13">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29" ht="19.5" customHeight="1">
       <c r="A29" t="s" s="14">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B29" t="s" s="18">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C29" t="s" s="16">
         <v>17</v>
@@ -3088,7 +3106,7 @@
         <v>0</v>
       </c>
       <c r="G29" t="s" s="16">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H29" s="19">
         <v>0</v>
@@ -3117,7 +3135,7 @@
     </row>
     <row r="30" ht="19.5" customHeight="1">
       <c r="A30" t="s" s="14">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B30" s="15">
         <v>0</v>
@@ -3164,7 +3182,7 @@
     </row>
     <row r="31" ht="19.5" customHeight="1">
       <c r="A31" t="s" s="14">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B31" s="15">
         <v>0</v>
@@ -3211,7 +3229,7 @@
     </row>
     <row r="32" ht="19.5" customHeight="1">
       <c r="A32" t="s" s="14">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B32" s="15">
         <v>20</v>
@@ -3253,12 +3271,12 @@
         <v>21</v>
       </c>
       <c r="O32" t="s" s="13">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="33" ht="19.5" customHeight="1">
       <c r="A33" t="s" s="14">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B33" s="15">
         <v>0</v>
@@ -3297,7 +3315,7 @@
         <v>20</v>
       </c>
       <c r="N33" t="s" s="16">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O33" t="s" s="13">
         <v>22</v>
@@ -3305,7 +3323,7 @@
     </row>
     <row r="34" ht="19.5" customHeight="1">
       <c r="A34" t="s" s="14">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B34" s="15">
         <v>0</v>
@@ -3343,7 +3361,7 @@
       <c r="M34" s="17">
         <v>0</v>
       </c>
-      <c r="N34" s="17">
+      <c r="N34" s="20">
         <v>0</v>
       </c>
       <c r="O34" s="22">
@@ -3351,38 +3369,98 @@
       </c>
     </row>
     <row r="35" ht="19.5" customHeight="1">
-      <c r="A35" s="23"/>
-      <c r="B35" s="24"/>
-      <c r="C35" s="25"/>
-      <c r="D35" s="25"/>
-      <c r="E35" s="25"/>
-      <c r="F35" s="25"/>
-      <c r="G35" s="25"/>
-      <c r="H35" s="25"/>
-      <c r="I35" s="25"/>
-      <c r="J35" s="25"/>
-      <c r="K35" s="25"/>
-      <c r="L35" s="25"/>
-      <c r="M35" s="25"/>
-      <c r="N35" s="25"/>
-      <c r="O35" s="26"/>
+      <c r="A35" t="s" s="14">
+        <v>81</v>
+      </c>
+      <c r="B35" s="15">
+        <v>7</v>
+      </c>
+      <c r="C35" t="s" s="16">
+        <v>17</v>
+      </c>
+      <c r="D35" t="s" s="16">
+        <v>17</v>
+      </c>
+      <c r="E35" t="s" s="16">
+        <v>17</v>
+      </c>
+      <c r="F35" s="17">
+        <v>0</v>
+      </c>
+      <c r="G35" s="17">
+        <v>0</v>
+      </c>
+      <c r="H35" s="17">
+        <v>1</v>
+      </c>
+      <c r="I35" s="17">
+        <v>0</v>
+      </c>
+      <c r="J35" s="17">
+        <v>0</v>
+      </c>
+      <c r="K35" s="17">
+        <v>0</v>
+      </c>
+      <c r="L35" t="s" s="16">
+        <v>19</v>
+      </c>
+      <c r="M35" t="s" s="16">
+        <v>20</v>
+      </c>
+      <c r="N35" t="s" s="21">
+        <v>40</v>
+      </c>
+      <c r="O35" t="s" s="13">
+        <v>82</v>
+      </c>
     </row>
     <row r="36" ht="19.5" customHeight="1">
-      <c r="A36" s="23"/>
-      <c r="B36" s="24"/>
-      <c r="C36" s="25"/>
-      <c r="D36" s="25"/>
-      <c r="E36" s="25"/>
-      <c r="F36" s="25"/>
-      <c r="G36" s="25"/>
-      <c r="H36" s="25"/>
-      <c r="I36" s="25"/>
-      <c r="J36" s="25"/>
-      <c r="K36" s="25"/>
-      <c r="L36" s="25"/>
-      <c r="M36" s="25"/>
-      <c r="N36" s="25"/>
-      <c r="O36" s="26"/>
+      <c r="A36" t="s" s="14">
+        <v>83</v>
+      </c>
+      <c r="B36" s="15">
+        <v>6</v>
+      </c>
+      <c r="C36" t="s" s="16">
+        <v>17</v>
+      </c>
+      <c r="D36" t="s" s="16">
+        <v>17</v>
+      </c>
+      <c r="E36" t="s" s="16">
+        <v>17</v>
+      </c>
+      <c r="F36" s="17">
+        <v>0</v>
+      </c>
+      <c r="G36" s="17">
+        <v>0</v>
+      </c>
+      <c r="H36" s="17">
+        <v>1</v>
+      </c>
+      <c r="I36" s="17">
+        <v>0</v>
+      </c>
+      <c r="J36" s="17">
+        <v>0</v>
+      </c>
+      <c r="K36" s="17">
+        <v>0</v>
+      </c>
+      <c r="L36" t="s" s="16">
+        <v>19</v>
+      </c>
+      <c r="M36" t="s" s="16">
+        <v>20</v>
+      </c>
+      <c r="N36" t="s" s="21">
+        <v>40</v>
+      </c>
+      <c r="O36" t="s" s="13">
+        <v>84</v>
+      </c>
     </row>
     <row r="37" ht="19.5" customHeight="1">
       <c r="A37" s="23"/>
@@ -3398,8 +3476,8 @@
       <c r="K37" s="25"/>
       <c r="L37" s="25"/>
       <c r="M37" s="25"/>
-      <c r="N37" s="25"/>
-      <c r="O37" s="26"/>
+      <c r="N37" s="26"/>
+      <c r="O37" s="27"/>
     </row>
     <row r="38" ht="19.5" customHeight="1">
       <c r="A38" s="23"/>
@@ -3416,7 +3494,7 @@
       <c r="L38" s="25"/>
       <c r="M38" s="25"/>
       <c r="N38" s="25"/>
-      <c r="O38" s="26"/>
+      <c r="O38" s="27"/>
     </row>
     <row r="39" ht="19.5" customHeight="1">
       <c r="A39" s="23"/>
@@ -3433,7 +3511,7 @@
       <c r="L39" s="25"/>
       <c r="M39" s="25"/>
       <c r="N39" s="25"/>
-      <c r="O39" s="26"/>
+      <c r="O39" s="27"/>
     </row>
     <row r="40" ht="19.5" customHeight="1">
       <c r="A40" s="23"/>
@@ -3450,7 +3528,7 @@
       <c r="L40" s="25"/>
       <c r="M40" s="25"/>
       <c r="N40" s="25"/>
-      <c r="O40" s="26"/>
+      <c r="O40" s="27"/>
     </row>
     <row r="41" ht="19.5" customHeight="1">
       <c r="A41" s="23"/>
@@ -3467,7 +3545,7 @@
       <c r="L41" s="25"/>
       <c r="M41" s="25"/>
       <c r="N41" s="25"/>
-      <c r="O41" s="26"/>
+      <c r="O41" s="27"/>
     </row>
     <row r="42" ht="19.5" customHeight="1">
       <c r="A42" s="23"/>
@@ -3484,7 +3562,7 @@
       <c r="L42" s="25"/>
       <c r="M42" s="25"/>
       <c r="N42" s="25"/>
-      <c r="O42" s="26"/>
+      <c r="O42" s="27"/>
     </row>
     <row r="43" ht="19.5" customHeight="1">
       <c r="A43" s="23"/>
@@ -3501,7 +3579,7 @@
       <c r="L43" s="25"/>
       <c r="M43" s="25"/>
       <c r="N43" s="25"/>
-      <c r="O43" s="26"/>
+      <c r="O43" s="27"/>
     </row>
     <row r="44" ht="19.5" customHeight="1">
       <c r="A44" s="23"/>
@@ -3518,7 +3596,7 @@
       <c r="L44" s="25"/>
       <c r="M44" s="25"/>
       <c r="N44" s="25"/>
-      <c r="O44" s="26"/>
+      <c r="O44" s="27"/>
     </row>
     <row r="45" ht="19.5" customHeight="1">
       <c r="A45" s="23"/>
@@ -3535,7 +3613,7 @@
       <c r="L45" s="25"/>
       <c r="M45" s="25"/>
       <c r="N45" s="25"/>
-      <c r="O45" s="26"/>
+      <c r="O45" s="27"/>
     </row>
     <row r="46" ht="19.5" customHeight="1">
       <c r="A46" s="23"/>
@@ -3552,7 +3630,7 @@
       <c r="L46" s="25"/>
       <c r="M46" s="25"/>
       <c r="N46" s="25"/>
-      <c r="O46" s="26"/>
+      <c r="O46" s="27"/>
     </row>
     <row r="47" ht="19.5" customHeight="1">
       <c r="A47" s="23"/>
@@ -3569,7 +3647,7 @@
       <c r="L47" s="25"/>
       <c r="M47" s="25"/>
       <c r="N47" s="25"/>
-      <c r="O47" s="26"/>
+      <c r="O47" s="27"/>
     </row>
     <row r="48" ht="19.5" customHeight="1">
       <c r="A48" s="23"/>
@@ -3586,7 +3664,7 @@
       <c r="L48" s="25"/>
       <c r="M48" s="25"/>
       <c r="N48" s="25"/>
-      <c r="O48" s="26"/>
+      <c r="O48" s="27"/>
     </row>
     <row r="49" ht="19.5" customHeight="1">
       <c r="A49" s="23"/>
@@ -3603,7 +3681,7 @@
       <c r="L49" s="25"/>
       <c r="M49" s="25"/>
       <c r="N49" s="25"/>
-      <c r="O49" s="26"/>
+      <c r="O49" s="27"/>
     </row>
     <row r="50" ht="19.5" customHeight="1">
       <c r="A50" s="23"/>
@@ -3620,7 +3698,7 @@
       <c r="L50" s="25"/>
       <c r="M50" s="25"/>
       <c r="N50" s="25"/>
-      <c r="O50" s="26"/>
+      <c r="O50" s="27"/>
     </row>
     <row r="51" ht="19.5" customHeight="1">
       <c r="A51" s="23"/>
@@ -3637,7 +3715,7 @@
       <c r="L51" s="25"/>
       <c r="M51" s="25"/>
       <c r="N51" s="25"/>
-      <c r="O51" s="26"/>
+      <c r="O51" s="27"/>
     </row>
     <row r="52" ht="19.5" customHeight="1">
       <c r="A52" s="23"/>
@@ -3654,7 +3732,7 @@
       <c r="L52" s="25"/>
       <c r="M52" s="25"/>
       <c r="N52" s="25"/>
-      <c r="O52" s="26"/>
+      <c r="O52" s="27"/>
     </row>
     <row r="53" ht="19.5" customHeight="1">
       <c r="A53" s="23"/>
@@ -3671,7 +3749,7 @@
       <c r="L53" s="25"/>
       <c r="M53" s="25"/>
       <c r="N53" s="25"/>
-      <c r="O53" s="26"/>
+      <c r="O53" s="27"/>
     </row>
     <row r="54" ht="19.5" customHeight="1">
       <c r="A54" s="23"/>
@@ -3688,7 +3766,7 @@
       <c r="L54" s="25"/>
       <c r="M54" s="25"/>
       <c r="N54" s="25"/>
-      <c r="O54" s="26"/>
+      <c r="O54" s="27"/>
     </row>
     <row r="55" ht="19.5" customHeight="1">
       <c r="A55" s="23"/>
@@ -3705,7 +3783,7 @@
       <c r="L55" s="25"/>
       <c r="M55" s="25"/>
       <c r="N55" s="25"/>
-      <c r="O55" s="26"/>
+      <c r="O55" s="27"/>
     </row>
     <row r="56" ht="19.5" customHeight="1">
       <c r="A56" s="23"/>
@@ -3722,7 +3800,7 @@
       <c r="L56" s="25"/>
       <c r="M56" s="25"/>
       <c r="N56" s="25"/>
-      <c r="O56" s="26"/>
+      <c r="O56" s="27"/>
     </row>
     <row r="57" ht="19.5" customHeight="1">
       <c r="A57" s="23"/>
@@ -3739,7 +3817,7 @@
       <c r="L57" s="25"/>
       <c r="M57" s="25"/>
       <c r="N57" s="25"/>
-      <c r="O57" s="26"/>
+      <c r="O57" s="27"/>
     </row>
     <row r="58" ht="19.5" customHeight="1">
       <c r="A58" s="23"/>
@@ -3756,7 +3834,7 @@
       <c r="L58" s="25"/>
       <c r="M58" s="25"/>
       <c r="N58" s="25"/>
-      <c r="O58" s="26"/>
+      <c r="O58" s="27"/>
     </row>
     <row r="59" ht="19.5" customHeight="1">
       <c r="A59" s="23"/>
@@ -3773,7 +3851,7 @@
       <c r="L59" s="25"/>
       <c r="M59" s="25"/>
       <c r="N59" s="25"/>
-      <c r="O59" s="26"/>
+      <c r="O59" s="27"/>
     </row>
     <row r="60" ht="19.5" customHeight="1">
       <c r="A60" s="23"/>
@@ -3790,7 +3868,7 @@
       <c r="L60" s="25"/>
       <c r="M60" s="25"/>
       <c r="N60" s="25"/>
-      <c r="O60" s="26"/>
+      <c r="O60" s="27"/>
     </row>
     <row r="61" ht="19.5" customHeight="1">
       <c r="A61" s="23"/>
@@ -3807,7 +3885,7 @@
       <c r="L61" s="25"/>
       <c r="M61" s="25"/>
       <c r="N61" s="25"/>
-      <c r="O61" s="26"/>
+      <c r="O61" s="27"/>
     </row>
     <row r="62" ht="19.5" customHeight="1">
       <c r="A62" s="23"/>
@@ -3824,7 +3902,7 @@
       <c r="L62" s="25"/>
       <c r="M62" s="25"/>
       <c r="N62" s="25"/>
-      <c r="O62" s="26"/>
+      <c r="O62" s="27"/>
     </row>
     <row r="63" ht="19.5" customHeight="1">
       <c r="A63" s="23"/>
@@ -3841,7 +3919,7 @@
       <c r="L63" s="25"/>
       <c r="M63" s="25"/>
       <c r="N63" s="25"/>
-      <c r="O63" s="26"/>
+      <c r="O63" s="27"/>
     </row>
     <row r="64" ht="19.5" customHeight="1">
       <c r="A64" s="23"/>
@@ -3858,7 +3936,7 @@
       <c r="L64" s="25"/>
       <c r="M64" s="25"/>
       <c r="N64" s="25"/>
-      <c r="O64" s="26"/>
+      <c r="O64" s="27"/>
     </row>
     <row r="65" ht="19.5" customHeight="1">
       <c r="A65" s="23"/>
@@ -3875,7 +3953,7 @@
       <c r="L65" s="25"/>
       <c r="M65" s="25"/>
       <c r="N65" s="25"/>
-      <c r="O65" s="26"/>
+      <c r="O65" s="27"/>
     </row>
     <row r="66" ht="19.5" customHeight="1">
       <c r="A66" s="23"/>
@@ -3892,7 +3970,7 @@
       <c r="L66" s="25"/>
       <c r="M66" s="25"/>
       <c r="N66" s="25"/>
-      <c r="O66" s="26"/>
+      <c r="O66" s="27"/>
     </row>
     <row r="67" ht="19.5" customHeight="1">
       <c r="A67" s="23"/>
@@ -3909,24 +3987,24 @@
       <c r="L67" s="25"/>
       <c r="M67" s="25"/>
       <c r="N67" s="25"/>
-      <c r="O67" s="26"/>
+      <c r="O67" s="27"/>
     </row>
     <row r="68" ht="19.5" customHeight="1">
-      <c r="A68" s="27"/>
-      <c r="B68" s="28"/>
-      <c r="C68" s="29"/>
-      <c r="D68" s="29"/>
-      <c r="E68" s="29"/>
-      <c r="F68" s="29"/>
-      <c r="G68" s="29"/>
-      <c r="H68" s="29"/>
-      <c r="I68" s="29"/>
-      <c r="J68" s="29"/>
-      <c r="K68" s="29"/>
-      <c r="L68" s="29"/>
-      <c r="M68" s="29"/>
-      <c r="N68" s="29"/>
-      <c r="O68" s="30"/>
+      <c r="A68" s="28"/>
+      <c r="B68" s="29"/>
+      <c r="C68" s="30"/>
+      <c r="D68" s="30"/>
+      <c r="E68" s="30"/>
+      <c r="F68" s="30"/>
+      <c r="G68" s="30"/>
+      <c r="H68" s="30"/>
+      <c r="I68" s="30"/>
+      <c r="J68" s="30"/>
+      <c r="K68" s="30"/>
+      <c r="L68" s="30"/>
+      <c r="M68" s="30"/>
+      <c r="N68" s="30"/>
+      <c r="O68" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
make addiu sign extended as it's need to be
</commit_message>
<xml_diff>
--- a/scripts/mips32_r2000_instruction_set.xlsx
+++ b/scripts/mips32_r2000_instruction_set.xlsx
@@ -94,22 +94,22 @@
     <t>addiu</t>
   </si>
   <si>
+    <t>addu</t>
+  </si>
+  <si>
+    <t>and</t>
+  </si>
+  <si>
+    <t>`ALUOp_AND</t>
+  </si>
+  <si>
+    <t>andi</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
     <t>`EXT_ZERO</t>
-  </si>
-  <si>
-    <t>addu</t>
-  </si>
-  <si>
-    <t>and</t>
-  </si>
-  <si>
-    <t>`ALUOp_AND</t>
-  </si>
-  <si>
-    <t>andi</t>
-  </si>
-  <si>
-    <t>c</t>
   </si>
   <si>
     <t>beq</t>
@@ -1996,7 +1996,7 @@
         <v>25</v>
       </c>
       <c r="M5" t="s" s="16">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="N5" t="s" s="16">
         <v>21</v>
@@ -2007,7 +2007,7 @@
     </row>
     <row r="6" ht="19.5" customHeight="1">
       <c r="A6" t="s" s="14">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B6" s="15">
         <v>0</v>
@@ -2054,7 +2054,7 @@
     </row>
     <row r="7" ht="19.5" customHeight="1">
       <c r="A7" t="s" s="14">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B7" s="15">
         <v>0</v>
@@ -2093,7 +2093,7 @@
         <v>20</v>
       </c>
       <c r="N7" t="s" s="16">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O7" t="s" s="13">
         <v>22</v>
@@ -2101,10 +2101,10 @@
     </row>
     <row r="8" ht="19.5" customHeight="1">
       <c r="A8" t="s" s="14">
+        <v>30</v>
+      </c>
+      <c r="B8" t="s" s="18">
         <v>31</v>
-      </c>
-      <c r="B8" t="s" s="18">
-        <v>32</v>
       </c>
       <c r="C8" t="s" s="16">
         <v>17</v>
@@ -2137,10 +2137,10 @@
         <v>25</v>
       </c>
       <c r="M8" t="s" s="16">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="N8" t="s" s="16">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O8" t="s" s="13">
         <v>22</v>
@@ -2513,7 +2513,7 @@
         <v>25</v>
       </c>
       <c r="M16" t="s" s="16">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="N16" t="s" s="16">
         <v>51</v>
@@ -2701,7 +2701,7 @@
         <v>25</v>
       </c>
       <c r="M20" t="s" s="16">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="N20" t="s" s="16">
         <v>56</v>
@@ -2842,7 +2842,7 @@
         <v>25</v>
       </c>
       <c r="M23" t="s" s="16">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="N23" t="s" s="16">
         <v>61</v>
@@ -2889,7 +2889,7 @@
         <v>19</v>
       </c>
       <c r="M24" t="s" s="16">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="N24" t="s" s="16">
         <v>61</v>

</xml_diff>